<commit_message>
Add through-Oct joined weather; convert HOBO lux by median
</commit_message>
<xml_diff>
--- a/data/weather_data/lab_weather_data/Lab_Weather_Joined_Interp30.xlsx
+++ b/data/weather_data/lab_weather_data/Lab_Weather_Joined_Interp30.xlsx
@@ -15833,10 +15833,10 @@
         <v>46213.66666666666</v>
       </c>
       <c r="B1101" t="n">
-        <v>27.01197276458061</v>
+        <v>27.19832036546537</v>
       </c>
       <c r="C1101" t="n">
-        <v>53.497314453125</v>
+        <v>53.582763671875</v>
       </c>
       <c r="D1101" t="n">
         <v>51.43097857142857</v>

</xml_diff>